<commit_message>
complete updated final project
</commit_message>
<xml_diff>
--- a/Documents/SCI_SE_9.ProjectTestReport.xlsx
+++ b/Documents/SCI_SE_9.ProjectTestReport.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="TestReportSprint1" sheetId="3" r:id="rId1"/>
@@ -114,10 +114,10 @@
     <t>Kiểm tra chức năng quên mật khẩu</t>
   </si>
   <si>
-    <t>Lấy lại mật khẩu</t>
+    <t>Đặt lại mật khẩu</t>
   </si>
   <si>
-    <t>Kiểm tra chức năng lấy lại mật khẩu</t>
+    <t>Kiểm tra chức năng đặt lại mật khẩu</t>
   </si>
   <si>
     <t>Danh sách việc làm</t>

</xml_diff>